<commit_message>
Corrige fichas de jogo e estatisticas da jornada
</commit_message>
<xml_diff>
--- a/public/templates/girabola_modelo_rodada_em_branco.xlsx
+++ b/public/templates/girabola_modelo_rodada_em_branco.xlsx
@@ -7,9 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jogos_Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eventos_Ocorrencias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clubes_Referencia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jogos_Resultados" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eventos_Ocorrencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estatisticas_Equipa" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbitragem" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Onzes_Convocatorias" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clubes_Referencia" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,12 +34,35 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFCC00"/>
+      <color rgb="000F1720"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="005A6672"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A2332"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="00FFCC00"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -78,15 +105,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -454,7 +492,335 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="118" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GIRABOLA — FICHEIRO PADRÃO DE JORNADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Modelo em branco · Liga Unitel Girabola</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>COMO USAR ESTE FICHEIRO</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Preencha uma jornada de cada vez. A coluna «Jornada» tem de estar preenchida em todas as linhas — linhas sem jornada são ignoradas pelo importador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Os nomes das equipas devem coincidir com a aba «Clubes_Referencia» (Nome_Curto, Nome_Oficial ou ID_Sistema são todos aceites).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Cada jogo é identificado pelo trio Jornada + Equipa_Casa + Equipa_Fora. Use sempre a mesma grafia em todas as abas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Depois de preencher, execute:  python3 scripts/import_rodada_excel.py &lt;caminho_do_ficheiro.xlsx&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>O importador gera public/templates/ultima_rodada_importada.json. Carregue esse JSON em Admin › Calendário › «Importar Dados» e depois «Guardar alterações».</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>REGRA EDITORIAL</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Célula vazia = dado ainda não publicado oficialmente. NUNCA preencher com estimativas, médias ou valores aproximados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Métricas ausentes na ficha oficial (posse, passes, remates…) devem ficar em branco: o site apresenta apenas o que foi publicado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Minuto por confirmar: deixar a célula «Minuto» vazia. O evento é publicado sem minuto, nunca com minuto inventado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ABAS DO FICHEIRO</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Jogos_Resultados</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Obrigatória. Agenda, resultado, estádio, transmissão, estado, árbitro principal, assistência e tempo útil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Eventos_Ocorrencias</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Golos, cartões amarelos/vermelhos e substituições. Uma linha por ocorrência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Estatisticas_Equipa</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Duas linhas por jogo (CASA e FORA). Só as métricas que constam da ficha oficial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Arbitragem</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Equipa de arbitragem completa. Uma linha por jogo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Onzes_Convocatorias</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Onze inicial e suplentes. Uma linha por atleta; Titular = SIM para o onze inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Clubes_Referencia</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Apenas consulta. Não editar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>VALORES ACEITES</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>finished (terminado) · scheduled (agendado) · live (em direto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Estado_Agenda</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>official (data confirmada) · provisional (data provisória)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Tipo_Evento</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>GOLO · AMARELO · VERMELHO · ADVERTENCIA · SUB</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Equipa_Infracao / Lado</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>CASA · FORA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Posicao</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>GK (guarda-redes) · DEF (defesa) · MID (médio) · FWD (avançado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Minuto</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Número (ex.: 63) ou compensação (ex.: 45+2, 90+5). Vazio se não confirmado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Data / Hora</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Data no formato AAAA-MM-DD e hora HH:MM (fuso de Luanda, +01:00).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -466,67 +832,402 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Jornada</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Data (AAAA-MM-DD)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Hora (HH:MM)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Equipa_Casa</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Golos_Casa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Golos_Fora</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Equipa_Fora</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Estadio</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Transmissao</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Status (finished/scheduled)</t>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Status (finished/scheduled/live)</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Estado_Agenda (official/provisional)</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Arbitro_Principal</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Assistencia</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Tempo_Util_Min</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>ID_Jogo (opcional)</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>Observacoes</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"finished,scheduled,live"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"official,provisional"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="29" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Casa</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Fora</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Minuto</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Tipo_Evento (GOLO/AMARELO/VERMELHO/ADVERTENCIA/SUB)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Infracao (CASA/FORA)</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Camisola</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Nome_Jogador</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Detalhe_Motivo</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Jogador_Saiu (apenas SUB)</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Assistencia_Golo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"GOLO,AMARELO,VERMELHO,SUB"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CASA,FORA"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Casa</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Fora</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Lado (CASA/FORA)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Posse_%</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Remates</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Remates_a_Baliza</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Cantos</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Faltas</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Foras_de_Jogo</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Amarelos</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Vermelhos</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Passes</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>Precisao_Passe_%</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Defesas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CASA,FORA"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Casa</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Equipa_Fora</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Arbitro_Principal</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Assistente_1</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Assistente_2</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Quarto_Arbitro</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -538,67 +1239,84 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="43" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Jornada</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Equipa_Casa</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Equipa_Fora</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Minuto</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo_Evento (GOLO/AMARELO/VERMELHO/SUB)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Equipa_Infracao (CASA/FORA)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Lado (CASA/FORA)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Camisola</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Nome_Jogador</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Detalhe_Motivo</t>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Posicao (GK/DEF/MID/FWD)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Titular (SIM/NAO)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Formacao</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Petro de Luanda,CD 1.º de Agosto,Sagrada Esperança,Desportivo da Lunda Sul,GD Interclube,Kabuscorp SC,Wiliete de Benguela,Bravos do Maquis,Desportivo da Huíla,Académica do Lobito,São Salvador,Estrela 1.º de Maio,Recreativo do Libolo,CR Caála,FC Luanda,FC Cabinda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CASA,FORA"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"GK,DEF,MID,FWD"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SIM,NAO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -614,460 +1332,460 @@
     <col width="35" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>ID_Sistema</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Nome_Oficial</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Nome_Curto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Sigla</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Estadio_Padrao</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>petro</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Petro Atlético de Luanda</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Petro de Luanda</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>PET</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Estádio 11 de Novembro</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>dago</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Clube Desportivo 1.º de Agosto</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>CD 1.º de Agosto</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>PRI</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Estádio França N’dalu</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>sagrada</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Grupo Desportivo Sagrada Esperança</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Sagrada Esperança</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>SAG</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Estádio Sagrada Esperança</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>lundasul</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Clube Desportivo da Lunda Sul</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Desportivo da Lunda Sul</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>LSU</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Estádio do Sagrada Esperança</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>interclube</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Grupo Desportivo Interclube</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>GD Interclube</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>INT</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Estádio 22 de Junho</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>kabuscorp</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Kabuscorp Sport Clube do Palanca</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Kabuscorp SC</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>KAB</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Estádio dos Coqueiros</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>wiliete</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Wiliete Sport Clube de Benguela</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Wiliete de Benguela</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>WIL</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Estádio Nacional de Ombaka</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>bravos</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Futebol Clube Bravos do Maquis</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Bravos do Maquis</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>BMA</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Estádio Mundunduleno</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>desphuila</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Clube Desportivo da Huíla</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Desportivo da Huíla</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>CDH</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Estádio da Tundavala</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>lobito</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Académica Petróleos do Lobito</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Académica do Lobito</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>ACA</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Estádio do Buraco</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>saosalvador</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>São Salvador Futebol Clube do Kongo</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>São Salvador</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>SSA</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Estádio Álvaro Buta</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>primeiromaio</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Estrela Clube 1.º de Maio de Benguela</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Estrela 1.º de Maio</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>MAI</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Estádio de São Filipe</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>libolo</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Clube Recreativo Desportivo do Libolo</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Recreativo do Libolo</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>LIB</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Estádio Municipal de Calulo</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>caala</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Clube Recreativo da Caála</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>CR Caála</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>CAA</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Estádio dos Mártires da Canhala</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>fcluanda</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Futebol Clube de Luanda</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>FC Luanda</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>FCL</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Estádio França N’dalu</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>cabinda</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Futebol Clube de Cabinda</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>FC Cabinda</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>CAB</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Estádio Vici António</t>
         </is>

</xml_diff>